<commit_message>
fix: update some basic function
</commit_message>
<xml_diff>
--- a/data/compare_compartment_anotation_with_and_without_filter.xlsx
+++ b/data/compare_compartment_anotation_with_and_without_filter.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D175"/>
+  <dimension ref="A1:D164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,10 +455,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2220</v>
+        <v>2225</v>
       </c>
       <c r="D2" t="n">
-        <v>1708</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="3">
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1186</v>
+        <v>1193</v>
       </c>
       <c r="D3" t="n">
         <v>1098</v>
@@ -483,14 +483,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>late endosome</t>
+          <t>membrane</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>29</v>
+        <v>1682</v>
       </c>
       <c r="D4" t="n">
-        <v>24</v>
+        <v>521</v>
       </c>
     </row>
     <row r="5">
@@ -499,15 +499,13 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Golgi apparatus</t>
+          <t>bounding membrane of organelle</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>257</v>
-      </c>
-      <c r="D5" t="n">
-        <v>104</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -519,7 +517,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6" t="inlineStr"/>
     </row>
@@ -529,14 +527,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>membrane</t>
+          <t>Golgi apparatus</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2069</v>
+        <v>260</v>
       </c>
       <c r="D7" t="n">
-        <v>455</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8">
@@ -545,14 +543,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>cytosol</t>
+          <t>endosome</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>786</v>
+        <v>151</v>
       </c>
       <c r="D8" t="n">
-        <v>544</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9">
@@ -561,14 +559,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>cytoplasm</t>
+          <t>late endosome</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2388</v>
+        <v>29</v>
       </c>
       <c r="D9" t="n">
-        <v>1816</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -577,14 +575,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>plasma membrane</t>
+          <t>cytosol</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>513</v>
+        <v>832</v>
       </c>
       <c r="D10" t="n">
-        <v>353</v>
+        <v>560</v>
       </c>
     </row>
     <row r="11">
@@ -593,14 +591,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>fungal-type vacuole membrane</t>
+          <t>cytoplasm</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>218</v>
+        <v>2480</v>
       </c>
       <c r="D11" t="n">
-        <v>212</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="12">
@@ -609,14 +607,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>extracellular region</t>
+          <t>plasma membrane</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>112</v>
+        <v>546</v>
       </c>
       <c r="D12" t="n">
-        <v>36</v>
+        <v>385</v>
       </c>
     </row>
     <row r="13">
@@ -625,14 +623,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>polysome</t>
+          <t>fungal-type vacuole membrane</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>29</v>
+        <v>216</v>
       </c>
       <c r="D13" t="n">
-        <v>27</v>
+        <v>211</v>
       </c>
     </row>
     <row r="14">
@@ -641,14 +639,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>fungal-type cell wall</t>
+          <t>extracellular region</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D14" t="n">
-        <v>91</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15">
@@ -657,14 +655,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum</t>
+          <t>fungal-type cell wall</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>656</v>
+        <v>115</v>
       </c>
       <c r="D15" t="n">
-        <v>550</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16">
@@ -673,13 +671,15 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum-Golgi intermediate compartment</t>
+          <t>endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>18</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
+        <v>398</v>
+      </c>
+      <c r="D16" t="n">
+        <v>134</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -687,14 +687,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>COPII-coated ER to Golgi transport vesicle</t>
+          <t>endoplasmic reticulum</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>27</v>
+        <v>669</v>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>555</v>
       </c>
     </row>
     <row r="18">
@@ -703,15 +703,13 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum membrane</t>
+          <t>endoplasmic reticulum-Golgi intermediate compartment</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>377</v>
-      </c>
-      <c r="D18" t="n">
-        <v>85</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -719,14 +717,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>integral component of membrane</t>
+          <t>COPII-coated ER to Golgi transport vesicle</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1505</v>
+        <v>27</v>
       </c>
       <c r="D19" t="n">
-        <v>460</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20">
@@ -735,14 +733,14 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>integral component of mitochondrial outer membrane</t>
+          <t>mitochondrial outer membrane</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>26</v>
+        <v>107</v>
       </c>
       <c r="D20" t="n">
-        <v>22</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21">
@@ -751,14 +749,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>mitochondrial outer membrane</t>
+          <t>nuclear membrane</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>102</v>
+        <v>69</v>
       </c>
       <c r="D21" t="n">
-        <v>83</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22">
@@ -767,14 +765,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>nuclear membrane</t>
+          <t>nucleoplasm</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="D22" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23">
@@ -787,7 +785,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="D23" t="inlineStr"/>
     </row>
@@ -797,14 +795,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>endosome</t>
+          <t>endosome membrane</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>147</v>
+        <v>71</v>
       </c>
       <c r="D24" t="n">
-        <v>89</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25">
@@ -813,14 +811,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>endosome membrane</t>
+          <t>cellular bud neck</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>67</v>
+        <v>195</v>
       </c>
       <c r="D25" t="n">
-        <v>9</v>
+        <v>184</v>
       </c>
     </row>
     <row r="26">
@@ -845,14 +843,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>cellular bud neck</t>
+          <t>mating projection tip</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>194</v>
+        <v>120</v>
       </c>
       <c r="D27" t="n">
-        <v>182</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28">
@@ -861,14 +859,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>mating projection tip</t>
+          <t>ascospore wall</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="D28" t="n">
-        <v>114</v>
+        <v>11</v>
       </c>
     </row>
     <row r="29">
@@ -877,15 +875,13 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ascospore wall</t>
+          <t>spore wall</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>11</v>
-      </c>
-      <c r="D29" t="n">
-        <v>11</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -913,10 +909,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D31" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32">
@@ -925,13 +921,15 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>spore wall</t>
+          <t>chromosome</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>7</v>
-      </c>
-      <c r="D32" t="inlineStr"/>
+        <v>155</v>
+      </c>
+      <c r="D32" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -943,10 +941,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D33" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34">
@@ -959,10 +957,10 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D34" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35">
@@ -971,14 +969,14 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>chromosome</t>
+          <t>P-body</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>140</v>
+        <v>57</v>
       </c>
       <c r="D35" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36">
@@ -987,14 +985,14 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>P-body</t>
+          <t>cellular bud</t>
         </is>
       </c>
       <c r="C36" t="n">
+        <v>68</v>
+      </c>
+      <c r="D36" t="n">
         <v>53</v>
-      </c>
-      <c r="D36" t="n">
-        <v>45</v>
       </c>
     </row>
     <row r="37">
@@ -1003,14 +1001,14 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>cellular bud</t>
+          <t>nucleolus</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>63</v>
+        <v>279</v>
       </c>
       <c r="D37" t="n">
-        <v>52</v>
+        <v>249</v>
       </c>
     </row>
     <row r="38">
@@ -1019,14 +1017,14 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>nucleolus</t>
+          <t>trans-Golgi network</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>273</v>
+        <v>42</v>
       </c>
       <c r="D38" t="n">
-        <v>246</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39">
@@ -1035,15 +1033,13 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>trans-Golgi network</t>
+          <t>vesicle</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>42</v>
-      </c>
-      <c r="D39" t="n">
-        <v>34</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -1051,13 +1047,15 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>vesicle</t>
+          <t>cell periphery</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>8</v>
-      </c>
-      <c r="D40" t="inlineStr"/>
+        <v>282</v>
+      </c>
+      <c r="D40" t="n">
+        <v>272</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -1065,14 +1063,14 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>cell periphery</t>
+          <t>U2-type catalytic step 1 spliceosome</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>274</v>
+        <v>13</v>
       </c>
       <c r="D41" t="n">
-        <v>272</v>
+        <v>12</v>
       </c>
     </row>
     <row r="42">
@@ -1081,14 +1079,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>U2-type catalytic step 1 spliceosome</t>
+          <t>U2-type catalytic step 2 spliceosome</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D42" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="43">
@@ -1097,14 +1095,14 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>U2-type catalytic step 2 spliceosome</t>
+          <t>cytoskeleton</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>11</v>
+        <v>152</v>
       </c>
       <c r="D43" t="n">
-        <v>8</v>
+        <v>47</v>
       </c>
     </row>
     <row r="44">
@@ -1117,10 +1115,10 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D44" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="45">
@@ -1129,14 +1127,14 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>cytoskeleton</t>
+          <t>cytoplasmic stress granule</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>155</v>
+        <v>98</v>
       </c>
       <c r="D45" t="n">
-        <v>43</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46">
@@ -1145,14 +1143,14 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>cytoplasmic stress granule</t>
+          <t>peroxisome</t>
         </is>
       </c>
       <c r="C46" t="n">
+        <v>134</v>
+      </c>
+      <c r="D46" t="n">
         <v>99</v>
-      </c>
-      <c r="D46" t="n">
-        <v>97</v>
       </c>
     </row>
     <row r="47">
@@ -1165,10 +1163,10 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="D47" t="n">
-        <v>91</v>
+        <v>120</v>
       </c>
     </row>
     <row r="48">
@@ -1184,7 +1182,7 @@
         <v>68</v>
       </c>
       <c r="D48" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="49">
@@ -1209,14 +1207,14 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>integral component of Golgi membrane</t>
+          <t>Golgi membrane</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>25</v>
+        <v>143</v>
       </c>
       <c r="D50" t="n">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51">
@@ -1225,14 +1223,14 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>integral component of endoplasmic reticulum membrane</t>
+          <t>mitochondrial matrix</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>67</v>
+        <v>134</v>
       </c>
       <c r="D51" t="n">
-        <v>46</v>
+        <v>80</v>
       </c>
     </row>
     <row r="52">
@@ -1241,14 +1239,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Golgi membrane</t>
+          <t>mitochondria-associated endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>138</v>
+        <v>11</v>
       </c>
       <c r="D52" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53">
@@ -1257,14 +1255,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>mitochondrial matrix</t>
+          <t>peroxisomal membrane</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>131</v>
+        <v>41</v>
       </c>
       <c r="D53" t="n">
-        <v>77</v>
+        <v>30</v>
       </c>
     </row>
     <row r="54">
@@ -1273,11 +1271,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>intracellular membrane-bounded organelle</t>
+          <t>side of membrane</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="D54" t="inlineStr"/>
     </row>
@@ -1287,14 +1285,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>peroxisome</t>
+          <t>nuclear pore</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>89</v>
+        <v>48</v>
       </c>
       <c r="D55" t="n">
-        <v>59</v>
+        <v>32</v>
       </c>
     </row>
     <row r="56">
@@ -1303,14 +1301,14 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>peroxisomal membrane</t>
+          <t>nuclear pore central transport channel</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="D56" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="57">
@@ -1319,13 +1317,15 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>cell cortex of cell tip</t>
+          <t>nuclear pore nuclear basket</t>
         </is>
       </c>
       <c r="C57" t="n">
+        <v>10</v>
+      </c>
+      <c r="D57" t="n">
         <v>9</v>
       </c>
-      <c r="D57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -1333,13 +1333,15 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>anchored component of membrane</t>
+          <t>condensed nuclear chromosome</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>64</v>
-      </c>
-      <c r="D58" t="inlineStr"/>
+        <v>25</v>
+      </c>
+      <c r="D58" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -1347,11 +1349,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>intrinsic component of membrane</t>
+          <t>microtubule cytoskeleton</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D59" t="inlineStr"/>
     </row>
@@ -1361,15 +1363,13 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>nuclear pore</t>
+          <t>cell tip</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>49</v>
-      </c>
-      <c r="D60" t="n">
-        <v>32</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="D60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -1377,14 +1377,14 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>nuclear pore central transport channel</t>
+          <t>nuclear envelope</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>14</v>
+        <v>78</v>
       </c>
       <c r="D61" t="n">
-        <v>13</v>
+        <v>66</v>
       </c>
     </row>
     <row r="62">
@@ -1393,14 +1393,14 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>nuclear pore nuclear basket</t>
+          <t>vacuolar membrane</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>9</v>
+        <v>182</v>
       </c>
       <c r="D62" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="63">
@@ -1409,14 +1409,14 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>condensed nuclear chromosome</t>
+          <t>vacuole</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>29</v>
+        <v>220</v>
       </c>
       <c r="D63" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
     </row>
     <row r="64">
@@ -1425,13 +1425,15 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>microtubule cytoskeleton</t>
+          <t>cytoplasmic vesicle</t>
         </is>
       </c>
       <c r="C64" t="n">
+        <v>57</v>
+      </c>
+      <c r="D64" t="n">
         <v>11</v>
       </c>
-      <c r="D64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -1439,11 +1441,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>cell tip</t>
+          <t>ER to Golgi transport vesicle membrane</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D65" t="inlineStr"/>
     </row>
@@ -1453,15 +1455,13 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>nuclear envelope</t>
+          <t>COPI-coated vesicle membrane</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>75</v>
-      </c>
-      <c r="D66" t="n">
-        <v>66</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="D66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -1469,13 +1469,15 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ER to Golgi transport vesicle membrane</t>
+          <t>Golgi trans cisterna</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>16</v>
-      </c>
-      <c r="D67" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="D67" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -1483,13 +1485,15 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>COPI-coated vesicle membrane</t>
+          <t>nuclear outer membrane</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>12</v>
-      </c>
-      <c r="D68" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="D68" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -1497,14 +1501,14 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>cytoplasmic vesicle</t>
+          <t>early endosome</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="D69" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="70">
@@ -1513,13 +1517,15 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>perinuclear endoplasmic reticulum</t>
+          <t>nucleus-vacuole junction</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>8</v>
-      </c>
-      <c r="D70" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="D70" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -1527,15 +1533,13 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Golgi trans cisterna</t>
+          <t>perinuclear endoplasmic reticulum</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>7</v>
-      </c>
-      <c r="D71" t="n">
-        <v>6</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="D71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -1543,13 +1547,15 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>nuclear outer membrane</t>
+          <t>nucleosome</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>6</v>
-      </c>
-      <c r="D72" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="D72" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -1557,14 +1563,14 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>early endosome</t>
+          <t>90S preribosome</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>18</v>
+        <v>80</v>
       </c>
       <c r="D73" t="n">
-        <v>13</v>
+        <v>79</v>
       </c>
     </row>
     <row r="74">
@@ -1573,14 +1579,14 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>nucleus-vacuole junction</t>
+          <t>cell cortex</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="D74" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
     </row>
     <row r="75">
@@ -1589,14 +1595,14 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>nucleosome</t>
+          <t>chromatin</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>11</v>
+        <v>110</v>
       </c>
       <c r="D75" t="n">
-        <v>8</v>
+        <v>81</v>
       </c>
     </row>
     <row r="76">
@@ -1605,15 +1611,13 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>nucleoplasm</t>
+          <t>periplasmic space</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>49</v>
-      </c>
-      <c r="D76" t="n">
-        <v>30</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="D76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -1621,14 +1625,14 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>90S preribosome</t>
+          <t>fungal-type vacuole</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>80</v>
+        <v>275</v>
       </c>
       <c r="D77" t="n">
-        <v>79</v>
+        <v>273</v>
       </c>
     </row>
     <row r="78">
@@ -1637,15 +1641,13 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>cell cortex</t>
+          <t>precatalytic spliceosome</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>45</v>
-      </c>
-      <c r="D78" t="n">
-        <v>27</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -1653,14 +1655,14 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>clathrin-coated vesicle</t>
+          <t>catalytic step 2 spliceosome</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D79" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
     </row>
     <row r="80">
@@ -1669,13 +1671,15 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>periplasmic space</t>
+          <t>ribosome</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>12</v>
-      </c>
-      <c r="D80" t="inlineStr"/>
+        <v>224</v>
+      </c>
+      <c r="D80" t="n">
+        <v>99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -1683,14 +1687,14 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>fungal-type vacuole</t>
+          <t>intracellular organelle</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>280</v>
+        <v>57</v>
       </c>
       <c r="D81" t="n">
-        <v>276</v>
+        <v>10</v>
       </c>
     </row>
     <row r="82">
@@ -1699,13 +1703,15 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>mitochondrial chromosome</t>
+          <t>cytoplasmic microtubule</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>6</v>
-      </c>
-      <c r="D82" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="D82" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -1713,13 +1719,15 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>precatalytic spliceosome</t>
+          <t>microtubule</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>16</v>
-      </c>
-      <c r="D83" t="inlineStr"/>
+        <v>57</v>
+      </c>
+      <c r="D83" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -1727,15 +1735,13 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>catalytic step 2 spliceosome</t>
+          <t>microtubule organizing center</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>23</v>
-      </c>
-      <c r="D84" t="n">
         <v>6</v>
       </c>
+      <c r="D84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -1743,15 +1749,13 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ribosome</t>
+          <t>clathrin-coated pit</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>228</v>
-      </c>
-      <c r="D85" t="n">
-        <v>104</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="D85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -1759,14 +1763,14 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>nuclear microtubule</t>
+          <t>membrane coat</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D86" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="87">
@@ -1775,11 +1779,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>cytoplasmic microtubule</t>
+          <t>cis-Golgi network</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D87" t="n">
         <v>15</v>
@@ -1791,15 +1795,13 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>microtubule</t>
+          <t>respirasome</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>57</v>
-      </c>
-      <c r="D88" t="n">
-        <v>24</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -1807,13 +1809,15 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>clathrin-coated pit</t>
+          <t>mitochondrial membrane</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>10</v>
-      </c>
-      <c r="D89" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="D89" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -1821,13 +1825,15 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>membrane coat</t>
+          <t>membrane raft</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>13</v>
-      </c>
-      <c r="D90" t="inlineStr"/>
+        <v>28</v>
+      </c>
+      <c r="D90" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -1835,14 +1841,14 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>cis-Golgi network</t>
+          <t>late endosome membrane</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D91" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="92">
@@ -1851,13 +1857,15 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>respirasome</t>
+          <t>phagophore assembly site</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>16</v>
-      </c>
-      <c r="D92" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="D92" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -1865,15 +1873,13 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>extrinsic component of membrane</t>
+          <t>autophagosome membrane</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>41</v>
-      </c>
-      <c r="D93" t="n">
-        <v>39</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="D93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -1881,11 +1887,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>mitochondrial membrane</t>
+          <t>vacuole-isolation membrane contact site</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>75</v>
+        <v>9</v>
       </c>
       <c r="D94" t="n">
         <v>9</v>
@@ -1897,14 +1903,14 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>membrane raft</t>
+          <t>nuclear periphery</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="D95" t="n">
-        <v>22</v>
+        <v>56</v>
       </c>
     </row>
     <row r="96">
@@ -1913,14 +1919,14 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>phagophore assembly site</t>
+          <t>site of polarized growth</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="D96" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
     </row>
     <row r="97">
@@ -1929,14 +1935,14 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>vacuole</t>
+          <t>mitochondrial nucleoid</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>197</v>
+        <v>24</v>
       </c>
       <c r="D97" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="98">
@@ -1945,14 +1951,14 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>vacuolar membrane</t>
+          <t>intracellular membrane-bounded organelle</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>171</v>
+        <v>68</v>
       </c>
       <c r="D98" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="99">
@@ -1961,11 +1967,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>vacuole-isolation membrane contact site</t>
+          <t>cell division site</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="D99" t="n">
         <v>9</v>
@@ -1977,14 +1983,14 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>nuclear periphery</t>
+          <t>cellular bud membrane</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>57</v>
+        <v>9</v>
       </c>
       <c r="D100" t="n">
-        <v>57</v>
+        <v>6</v>
       </c>
     </row>
     <row r="101">
@@ -1993,14 +1999,14 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>site of polarized growth</t>
+          <t>eisosome</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D101" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="102">
@@ -2009,15 +2015,13 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>mitochondrial nucleoid</t>
+          <t>cytoplasmic vesicle membrane</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>24</v>
-      </c>
-      <c r="D102" t="n">
-        <v>24</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="D102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -2025,15 +2029,13 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>extrinsic component of fungal-type vacuolar membrane</t>
+          <t>cell septum</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>7</v>
-      </c>
-      <c r="D103" t="n">
-        <v>7</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="D103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -2041,15 +2043,13 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>integral component of plasma membrane</t>
+          <t>transport vesicle</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>56</v>
-      </c>
-      <c r="D104" t="n">
-        <v>28</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="D104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
@@ -2057,15 +2057,13 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>cellular bud membrane</t>
+          <t>cytoplasmic side of plasma membrane</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>9</v>
-      </c>
-      <c r="D105" t="n">
-        <v>6</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="D105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
@@ -2073,15 +2071,13 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>eisosome</t>
+          <t>cell surface</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>21</v>
-      </c>
-      <c r="D106" t="n">
-        <v>21</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="D106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
@@ -2089,13 +2085,15 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>cell septum</t>
+          <t>nuclear outer membrane-endoplasmic reticulum membrane network</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>7</v>
-      </c>
-      <c r="D107" t="inlineStr"/>
+        <v>11</v>
+      </c>
+      <c r="D107" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
@@ -2103,13 +2101,15 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>cytoplasmic vesicle membrane</t>
+          <t>cortical endoplasmic reticulum</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>15</v>
-      </c>
-      <c r="D108" t="inlineStr"/>
+        <v>27</v>
+      </c>
+      <c r="D108" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -2117,14 +2117,14 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>transport vesicle</t>
+          <t>replication fork</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D109" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="110">
@@ -2133,13 +2133,15 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>cell surface</t>
+          <t>cell wall-bounded periplasmic space</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>18</v>
-      </c>
-      <c r="D110" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="D110" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -2147,14 +2149,14 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>nuclear outer membrane-endoplasmic reticulum membrane network</t>
+          <t>exocyst</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="D111" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="112">
@@ -2163,14 +2165,14 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>late endosome membrane</t>
+          <t>U2-type prespliceosome</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="D112" t="n">
-        <v>7</v>
+        <v>29</v>
       </c>
     </row>
     <row r="113">
@@ -2179,14 +2181,14 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>cortical endoplasmic reticulum</t>
+          <t>mitochondrial ribosome</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="D113" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
     </row>
     <row r="114">
@@ -2195,14 +2197,14 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>replication fork</t>
+          <t>vacuolar proton-transporting V-type ATPase, V1 domain</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D114" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="115">
@@ -2211,14 +2213,14 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>cell wall-bounded periplasmic space</t>
+          <t>vacuole-mitochondrion membrane contact site</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D115" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="116">
@@ -2227,15 +2229,13 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>exocyst</t>
+          <t>phagophore assembly site membrane</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>9</v>
-      </c>
-      <c r="D116" t="n">
-        <v>8</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="D116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -2243,14 +2243,14 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>U2-type prespliceosome</t>
+          <t>cellular bud neck septin ring</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D117" t="n">
-        <v>29</v>
+        <v>14</v>
       </c>
     </row>
     <row r="118">
@@ -2259,11 +2259,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>mitochondrial ribosome</t>
+          <t>cellular bud neck septin collar</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D118" t="n">
         <v>7</v>
@@ -2275,15 +2275,13 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>vacuolar proton-transporting V-type ATPase, V1 domain</t>
+          <t>vacuolar lumen</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>7</v>
-      </c>
-      <c r="D119" t="n">
-        <v>7</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="D119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -2291,14 +2289,14 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>vacuole-mitochondrion membrane contact site</t>
+          <t>fungal-type vacuole lumen</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D120" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="121">
@@ -2307,11 +2305,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>phagophore assembly site membrane</t>
+          <t>intracellular non-membrane-bounded organelle</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D121" t="inlineStr"/>
     </row>
@@ -2321,14 +2319,14 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>cellular bud neck septin ring</t>
+          <t>perinuclear region of cytoplasm</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D122" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="123">
@@ -2337,14 +2335,14 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>cellular bud neck septin collar</t>
+          <t>Golgi medial cisterna</t>
         </is>
       </c>
       <c r="C123" t="n">
         <v>7</v>
       </c>
       <c r="D123" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="124">
@@ -2353,14 +2351,14 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>fungal-type vacuole lumen</t>
+          <t>peroxisomal matrix</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D124" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="125">
@@ -2369,14 +2367,14 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>integral component of fungal-type vacuolar membrane</t>
+          <t>endoplasmic reticulum lumen</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D125" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="126">
@@ -2385,7 +2383,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>kinetochore microtubule</t>
+          <t>mitochondrial crista junction</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -2401,14 +2399,14 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>integral component of peroxisomal membrane</t>
+          <t>site of double-strand break</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D127" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="128">
@@ -2417,14 +2415,14 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>perinuclear region of cytoplasm</t>
+          <t>euchromatin</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D128" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="129">
@@ -2433,14 +2431,14 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Golgi medial cisterna</t>
+          <t>nuclear chromosome</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D129" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="130">
@@ -2449,14 +2447,14 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>peroxisomal matrix</t>
+          <t>cellular bud neck contractile ring</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D130" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="131">
@@ -2465,15 +2463,13 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum lumen</t>
+          <t>septin ring</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>16</v>
-      </c>
-      <c r="D131" t="n">
-        <v>9</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="D131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
@@ -2481,14 +2477,14 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>integral component of mitochondrial membrane</t>
+          <t>nuclear replication fork</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D132" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="133">
@@ -2497,14 +2493,14 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>extrinsic component of mitochondrial inner membrane</t>
+          <t>mating projection base</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D133" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
     </row>
     <row r="134">
@@ -2513,14 +2509,14 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>mitochondrial crista junction</t>
+          <t>mating projection</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D134" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="135">
@@ -2529,15 +2525,13 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>site of double-strand break</t>
+          <t>endocytic vesicle</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>13</v>
-      </c>
-      <c r="D135" t="n">
-        <v>9</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="D135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
@@ -2545,15 +2539,13 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>transcriptionally active chromatin</t>
+          <t>extracellular space</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>8</v>
-      </c>
-      <c r="D136" t="n">
-        <v>8</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="D136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
@@ -2561,14 +2553,14 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>nuclear chromosome</t>
+          <t>Golgi cis cisterna</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D137" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="138">
@@ -2577,14 +2569,14 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>COPI-coated vesicle</t>
+          <t>vacuolar proton-transporting V-type ATPase, V0 domain</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D138" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="139">
@@ -2593,14 +2585,14 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>cellular bud neck contractile ring</t>
+          <t>cytosolic ribosome</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D139" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="140">
@@ -2609,14 +2601,14 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>chromatin</t>
+          <t>COPI vesicle coat</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>87</v>
+        <v>8</v>
       </c>
       <c r="D140" t="n">
-        <v>76</v>
+        <v>8</v>
       </c>
     </row>
     <row r="141">
@@ -2625,13 +2617,15 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>septin ring</t>
+          <t>polarisome</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>12</v>
-      </c>
-      <c r="D141" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="D141" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
@@ -2639,15 +2633,13 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>nuclear replication fork</t>
+          <t>clathrin-coated vesicle membrane</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>16</v>
-      </c>
-      <c r="D142" t="n">
-        <v>16</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="D142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
@@ -2655,15 +2647,13 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>cell division site</t>
+          <t>early endosome membrane</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>24</v>
-      </c>
-      <c r="D143" t="n">
-        <v>9</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="D143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
@@ -2671,14 +2661,14 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>mating projection base</t>
+          <t>condensed chromosome, centromeric region</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D144" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="145">
@@ -2687,14 +2677,14 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>mating projection</t>
+          <t>proteasome storage granule</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D145" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="146">
@@ -2703,11 +2693,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>extrinsic component of plasma membrane</t>
+          <t>COPII vesicle coat</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D146" t="n">
         <v>7</v>
@@ -2719,11 +2709,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>extracellular space</t>
+          <t>endoplasmic reticulum exit site</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D147" t="inlineStr"/>
     </row>
@@ -2733,13 +2723,15 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>vacuolar lumen</t>
+          <t>cellular bud scar</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>7</v>
-      </c>
-      <c r="D148" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="D148" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
@@ -2747,15 +2739,13 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Golgi cis cisterna</t>
+          <t>cell cortex of cell tip</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>6</v>
-      </c>
-      <c r="D149" t="n">
-        <v>6</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="D149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
@@ -2763,15 +2753,13 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>vacuolar proton-transporting V-type ATPase, V0 domain</t>
+          <t>clathrin-coated vesicle</t>
         </is>
       </c>
       <c r="C150" t="n">
         <v>7</v>
       </c>
-      <c r="D150" t="n">
-        <v>7</v>
-      </c>
+      <c r="D150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
@@ -2779,13 +2767,15 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>proton-transporting V-type ATPase, V0 domain</t>
+          <t>endoplasmic reticulum tubular network</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>7</v>
-      </c>
-      <c r="D151" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="D151" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
@@ -2793,14 +2783,14 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>proteasome storage granule</t>
+          <t>rDNA heterochromatin</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D152" t="n">
-        <v>25</v>
+        <v>11</v>
       </c>
     </row>
     <row r="153">
@@ -2809,14 +2799,14 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>integral component of mitochondrial inner membrane</t>
+          <t>nuclear inner membrane</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="D153" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="154">
@@ -2825,13 +2815,15 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>cell projection</t>
+          <t>COP9 signalosome</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>8</v>
-      </c>
-      <c r="D154" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="D154" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
@@ -2839,15 +2831,13 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>COPI vesicle coat</t>
+          <t>membrane-bounded organelle</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>8</v>
-      </c>
-      <c r="D155" t="n">
-        <v>8</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="D155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
@@ -2855,14 +2845,14 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>polarisome</t>
+          <t>nuclear pore cytoplasmic filaments</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D156" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="157">
@@ -2871,7 +2861,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>clathrin-coated vesicle membrane</t>
+          <t>multivesicular body</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -2885,13 +2875,15 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>early endosome membrane</t>
+          <t>nuclear pore outer ring</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>8</v>
-      </c>
-      <c r="D158" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="D158" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
@@ -2899,14 +2891,14 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>condensed chromosome, centromeric region</t>
+          <t>signal recognition particle, endoplasmic reticulum targeting</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D159" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="160">
@@ -2915,13 +2907,15 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum exit site</t>
+          <t>phagophore</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>8</v>
-      </c>
-      <c r="D160" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="D160" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
@@ -2929,15 +2923,13 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>COPII vesicle coat</t>
+          <t>clathrin vesicle coat</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>8</v>
-      </c>
-      <c r="D161" t="n">
         <v>7</v>
       </c>
+      <c r="D161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
@@ -2945,14 +2937,14 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>cellular bud scar</t>
+          <t>matrix side of mitochondrial inner membrane</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D162" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="163">
@@ -2961,14 +2953,14 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum tubular network</t>
+          <t>mitochondrial envelope</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D163" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="164">
@@ -2977,185 +2969,13 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>rDNA heterochromatin</t>
+          <t>cellular bud neck split septin rings</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D164" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="1" t="n">
-        <v>163</v>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>nuclear inner membrane</t>
-        </is>
-      </c>
-      <c r="C165" t="n">
-        <v>16</v>
-      </c>
-      <c r="D165" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="1" t="n">
-        <v>164</v>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>COP9 signalosome</t>
-        </is>
-      </c>
-      <c r="C166" t="n">
-        <v>7</v>
-      </c>
-      <c r="D166" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="1" t="n">
-        <v>165</v>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>nuclear pore cytoplasmic filaments</t>
-        </is>
-      </c>
-      <c r="C167" t="n">
-        <v>9</v>
-      </c>
-      <c r="D167" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="1" t="n">
-        <v>166</v>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>multivesicular body</t>
-        </is>
-      </c>
-      <c r="C168" t="n">
-        <v>9</v>
-      </c>
-      <c r="D168" t="inlineStr"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="1" t="n">
-        <v>167</v>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>nuclear pore outer ring</t>
-        </is>
-      </c>
-      <c r="C169" t="n">
-        <v>7</v>
-      </c>
-      <c r="D169" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="1" t="n">
-        <v>168</v>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>signal recognition particle, endoplasmic reticulum targeting</t>
-        </is>
-      </c>
-      <c r="C170" t="n">
-        <v>6</v>
-      </c>
-      <c r="D170" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="1" t="n">
-        <v>169</v>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>cytosolic ribosome</t>
-        </is>
-      </c>
-      <c r="C171" t="n">
-        <v>8</v>
-      </c>
-      <c r="D171" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="1" t="n">
-        <v>170</v>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>phagophore</t>
-        </is>
-      </c>
-      <c r="C172" t="n">
-        <v>7</v>
-      </c>
-      <c r="D172" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="1" t="n">
-        <v>171</v>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>clathrin vesicle coat</t>
-        </is>
-      </c>
-      <c r="C173" t="n">
-        <v>6</v>
-      </c>
-      <c r="D173" t="inlineStr"/>
-    </row>
-    <row r="174">
-      <c r="A174" s="1" t="n">
-        <v>172</v>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>mitochondrial envelope</t>
-        </is>
-      </c>
-      <c r="C174" t="n">
-        <v>12</v>
-      </c>
-      <c r="D174" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="1" t="n">
-        <v>173</v>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>cellular bud neck split septin rings</t>
-        </is>
-      </c>
-      <c r="C175" t="n">
-        <v>6</v>
-      </c>
-      <c r="D175" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>